<commit_message>
Update feedback status tracking to include verification pending items
Modify the Python script to handle a new "Done — needs verification" status, update the consolidated workbook, and adjust the markdown report to reflect this change.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ee3bcdd9-84c0-4f0e-84c9-ead7b1026251
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a39e11a9-bfe3-4dd9-8d21-15cf9808d9f4
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/5ad98f17-de16-4057-90b7-eb39bee4dbc3/ee3bcdd9-84c0-4f0e-84c9-ead7b1026251/CgqJueA
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
+++ b/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
@@ -1616,7 +1616,7 @@
       </c>
       <c r="L13" s="15" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Done — needs verification</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>Fase 5 explicitly lists 'seguimiento de contratistas, cumplimiento de contratos, incumplimientos' as deliverables to the client. Contractor monitoring is a core V1 construction-phase feature. | Done in #75 + #62 (Contractor Estimate Rollup on the project report).</t>
+          <t>Fase 5 explicitly lists 'seguimiento de contratistas, cumplimiento de contratos, incumplimientos' as deliverables to the client. Contractor monitoring is a core V1 construction-phase feature. | Likely closed by #62 + #75 (Contractor Estimate Rollup on the project report); needs PM eyes-on confirmation that the consolidated view matches the original ask.</t>
         </is>
       </c>
     </row>
@@ -6500,7 +6500,9 @@
           <t>In Progress</t>
         </is>
       </c>
-      <c r="B18" s="24" t="inlineStr"/>
+      <c r="B18" s="24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="34" t="inlineStr">
@@ -6509,7 +6511,7 @@
         </is>
       </c>
       <c r="B19" s="24" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -6518,7 +6520,9 @@
           <t>Needs Spec</t>
         </is>
       </c>
-      <c r="B20" s="24" t="inlineStr"/>
+      <c r="B20" s="24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="36" t="inlineStr">
@@ -6530,7 +6534,16 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22"/>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Done — needs verification</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+    </row>
     <row r="23"/>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="26" t="inlineStr">

</xml_diff>

<commit_message>
Integrate Asana for bidirectional task and activity synchronization
Implements a comprehensive Asana integration, enabling bidirectional synchronization of project activities, lead acceptance task creation, and new logging endpoints for site visits and client interactions. Includes API endpoints, dashboard components, and backend logic for configuration, status checks, and sync log management.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ee3bcdd9-84c0-4f0e-84c9-ead7b1026251
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b6a7dc88-c247-42fd-89cb-97d5edbedfbe
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/5ad98f17-de16-4057-90b7-eb39bee4dbc3/ee3bcdd9-84c0-4f0e-84c9-ead7b1026251/SIfCYDi
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
+++ b/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
@@ -4636,7 +4636,7 @@
       </c>
       <c r="L60" s="14" t="inlineStr">
         <is>
-          <t>Needs Decision</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M60" s="8" t="inlineStr">
@@ -4646,7 +4646,7 @@
       </c>
       <c r="N60" s="10" t="inlineStr">
         <is>
-          <t>Fase 1 defines a 'CRM ligero integrado' and 'Notificación de tareas en ASANA'. Clarifying the CRM vs. Asana relationship is a V1 product decision that must be resolved before the CRM can be used.</t>
+          <t>Fase 1 defines a 'CRM ligero integrado' and 'Notificación de tareas en ASANA'. Clarifying the CRM vs. Asana relationship is a V1 product decision that must be resolved before the CRM can be used. | Done in #127 (real bidirectional Asana integration): leads now create real Asana tasks via lib/asana-client.createTask() with graceful fallback when the connector is unavailable; dashboard activity (uploads, photos, site visits, client interactions, phase changes, contract signed) is mirrored into Asana via lib/asana-sync.ts; admin-only Settings → Asana panel for connect/configure/sync log/retry; project_team_actions modals for site visits, client interactions, and Asana task linking.</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6511,7 @@
         </is>
       </c>
       <c r="B19" s="24" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -6531,7 +6531,7 @@
         </is>
       </c>
       <c r="B21" s="24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Update application to send real emails for project events
Implement transactional email sending using Resend for various project-related events, including signature requests, approvals, and phase changes. This includes adding new API endpoints, updating UI components to trigger these emails, and enhancing test coverage for mailer functionality.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ee3bcdd9-84c0-4f0e-84c9-ead7b1026251
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 14681290-da22-46a9-9d9d-160798276902
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/5ad98f17-de16-4057-90b7-eb39bee4dbc3/ee3bcdd9-84c0-4f0e-84c9-ead7b1026251/X8RiQjs
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
+++ b/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
@@ -5016,7 +5016,7 @@
       </c>
       <c r="L66" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M66" s="8" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="N66" s="10" t="inlineStr">
         <is>
-          <t>The workflow includes automated follow-up and notification emails across multiple phases (Fase 1 lead capture, Fase 2 contract, Fase 4 permit signatures). Email notifications are a V1 automation requirement.</t>
+          <t>The workflow includes automated follow-up and notification emails across multiple phases (Fase 1 lead capture, Fase 2 contract, Fase 4 permit signatures). Email notifications are a V1 automation requirement. | Done in #102 (Real signature handoff emails): permits-panel.tsx adds a 'Request signature' / 'Solicitar firma' button for staff that POSTs to a new dedupe-protected /projects/:id/request-signature/:signatureId endpoint and dispatches a bilingual Resend-backed email; the existing /sign endpoint now also emails the team a signature-completed notice; the previously-simulated Pre-Design kickoff, decline-notify-team, and proposal-acceptance emails are now real sends. All five flows isolate failures (mutation succeeds, email_failed activity row + UI toast surfaced) and are covered by node:test fixtures in artifacts/api-server/src/routes/__tests__/signature-emails.test.ts.</t>
         </is>
       </c>
     </row>
@@ -6491,7 +6491,7 @@
         </is>
       </c>
       <c r="B17" s="24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
@@ -6511,7 +6511,7 @@
         </is>
       </c>
       <c r="B19" s="24" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">

</xml_diff>

<commit_message>
Update project status with client activity log details
Update report and script to reflect the completion of the client-side audit log feature, including backend and frontend changes and existing test coverage.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ee3bcdd9-84c0-4f0e-84c9-ead7b1026251
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: cfd3ebdd-9307-48ef-98ef-c4e247f3c527
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/5ad98f17-de16-4057-90b7-eb39bee4dbc3/ee3bcdd9-84c0-4f0e-84c9-ead7b1026251/X8RiQjs
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
+++ b/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
@@ -1698,7 +1698,7 @@
       </c>
       <c r="N14" s="10" t="inlineStr">
         <is>
-          <t>The workflow does not include an audit log module. This is a compliance/governance feature that adds significant backend complexity beyond the V1 portal scope. Defer to V2. | Done in #61 hardening + verified 2026-05 (Task #156): client-side audit log shipped — backend GET /api/projects/:id/audit-log accepts the client role behind enforceClientOwnership with a `?clientOnly=true` filter (artifacts/api-server/src/routes/projects.ts ~L2386), and the bilingual ClientActivityCard is mounted on the client project page (artifacts/konti-dashboard/src/components/client-activity-card.tsx + project-detail.tsx ~L1721) with a Show-all / Client-only toggle. Non-owner 403 + owner 200 paths covered by client-ownership.test.ts L382-L420.</t>
+          <t>The workflow does not include an audit log module. This is a compliance/governance feature that adds significant backend complexity beyond the V1 portal scope. Defer to V2. | Done in #61 hardening + verified 2026-05 (Task #156): client-side audit log shipped — backend GET /api/projects/:id/audit-log accepts the client role behind enforceClientOwnership with a `?clientOnly=true` filter (artifacts/api-server/src/routes/projects.ts ~L2386), and the bilingual ClientActivityCard is mounted on the project detail page (artifacts/konti-dashboard/src/components/client-activity-card.tsx + project-detail.tsx ~L1721) with a Show-all / Client-only toggle. Non-owner 403 + owner 200 paths covered by client-ownership.test.ts L382-L420 (pre-existing — no new test was needed in this task).</t>
         </is>
       </c>
     </row>
@@ -5540,7 +5540,7 @@
       </c>
       <c r="N6" s="10" t="inlineStr">
         <is>
-          <t>The workflow does not include an audit log module. This is a compliance/governance feature that adds significant backend complexity beyond the V1 portal scope. Defer to V2. | Done in #61 hardening + verified 2026-05 (Task #156): client-side audit log shipped — backend GET /api/projects/:id/audit-log accepts the client role behind enforceClientOwnership with a `?clientOnly=true` filter (artifacts/api-server/src/routes/projects.ts ~L2386), and the bilingual ClientActivityCard is mounted on the client project page (artifacts/konti-dashboard/src/components/client-activity-card.tsx + project-detail.tsx ~L1721) with a Show-all / Client-only toggle. Non-owner 403 + owner 200 paths covered by client-ownership.test.ts L382-L420.</t>
+          <t>The workflow does not include an audit log module. This is a compliance/governance feature that adds significant backend complexity beyond the V1 portal scope. Defer to V2. | Done in #61 hardening + verified 2026-05 (Task #156): client-side audit log shipped — backend GET /api/projects/:id/audit-log accepts the client role behind enforceClientOwnership with a `?clientOnly=true` filter (artifacts/api-server/src/routes/projects.ts ~L2386), and the bilingual ClientActivityCard is mounted on the project detail page (artifacts/konti-dashboard/src/components/client-activity-card.tsx + project-detail.tsx ~L1721) with a Show-all / Client-only toggle. Non-owner 403 + owner 200 paths covered by client-ownership.test.ts L382-L420 (pre-existing — no new test was needed in this task).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update task status and documentation for Asana integration
Update MAP entries in `reconcile_feedback_status.py` and markdown reports to reflect completed Asana integration tasks, including changes to EN|ES comment formatting in `feedback-status-reconciled.md`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ee3bcdd9-84c0-4f0e-84c9-ead7b1026251
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4916796c-52fc-445d-b870-3ed821907a8f
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/5ad98f17-de16-4057-90b7-eb39bee4dbc3/ee3bcdd9-84c0-4f0e-84c9-ead7b1026251/X8RiQjs
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
+++ b/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
@@ -4718,7 +4718,7 @@
       </c>
       <c r="N61" s="6" t="inlineStr">
         <is>
-          <t>The workflow shows 'Notificación de tareas en ASANA' as an internal automation, but full bidirectional Asana API integration (template-driven project creation) is a complex third-party dependency. Basic ASANA notification is V1; full template automation is V2. | Done + verified 2026-05 (Task #157): Asana project creation from accepted leads shipped via #127. POST /api/leads/:id/accept calls lib/asana-client.createTask with the configured workspace + board (artifacts/api-server/src/routes/leads.ts L212-L242), synthesising the Asana task name as `${contactName} — ${projectType} (${location})` and a notes block with source/budget/land/contact/free-form notes; the new dashboard project is linked back via asanaGid and ongoing activity (uploads, photos, site visits, client interactions, phase changes, contract signed, proposal/change-order decisions, etc.) is mirrored as bilingual EN|ES comments on that task by lib/asana-sync.ts (SYNC_TYPES). Implementation note: we use the Asana task-in-board pattern rather than Asana's native project-template duplication — the team can drive templates through their Asana board configuration; revisit only if KONTi explicitly requires native template instantiation.</t>
+          <t>The workflow shows 'Notificación de tareas en ASANA' as an internal automation, but full bidirectional Asana API integration (template-driven project creation) is a complex third-party dependency. Basic ASANA notification is V1; full template automation is V2. | Done + verified 2026-05 (Task #157): Asana project creation from accepted leads shipped via #127. POST /api/leads/:id/accept calls lib/asana-client.createTask with the configured workspace + board (artifacts/api-server/src/routes/leads.ts L212-L242), synthesising the Asana task name as `${contactName} — ${projectType} (${location})` and a notes block with source/budget/land/contact/free-form notes; the new dashboard project is linked back via asanaGid and ongoing activity (uploads, photos, site visits, client interactions, phase changes, contract signed, proposal/change-order decisions, etc.) is mirrored as bilingual EN/ES comments on that task by lib/asana-sync.ts (SYNC_TYPES). Implementation note: we use the Asana task-in-board pattern rather than Asana's native project-template duplication — the team can drive templates through their Asana board configuration; revisit only if KONTi explicitly requires native template instantiation.</t>
         </is>
       </c>
     </row>
@@ -6216,7 +6216,7 @@
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
-          <t>The workflow shows 'Notificación de tareas en ASANA' as an internal automation, but full bidirectional Asana API integration (template-driven project creation) is a complex third-party dependency. Basic ASANA notification is V1; full template automation is V2. | Done + verified 2026-05 (Task #157): Asana project creation from accepted leads shipped via #127. POST /api/leads/:id/accept calls lib/asana-client.createTask with the configured workspace + board (artifacts/api-server/src/routes/leads.ts L212-L242), synthesising the Asana task name as `${contactName} — ${projectType} (${location})` and a notes block with source/budget/land/contact/free-form notes; the new dashboard project is linked back via asanaGid and ongoing activity (uploads, photos, site visits, client interactions, phase changes, contract signed, proposal/change-order decisions, etc.) is mirrored as bilingual EN|ES comments on that task by lib/asana-sync.ts (SYNC_TYPES). Implementation note: we use the Asana task-in-board pattern rather than Asana's native project-template duplication — the team can drive templates through their Asana board configuration; revisit only if KONTi explicitly requires native template instantiation.</t>
+          <t>The workflow shows 'Notificación de tareas en ASANA' as an internal automation, but full bidirectional Asana API integration (template-driven project creation) is a complex third-party dependency. Basic ASANA notification is V1; full template automation is V2. | Done + verified 2026-05 (Task #157): Asana project creation from accepted leads shipped via #127. POST /api/leads/:id/accept calls lib/asana-client.createTask with the configured workspace + board (artifacts/api-server/src/routes/leads.ts L212-L242), synthesising the Asana task name as `${contactName} — ${projectType} (${location})` and a notes block with source/budget/land/contact/free-form notes; the new dashboard project is linked back via asanaGid and ongoing activity (uploads, photos, site visits, client interactions, phase changes, contract signed, proposal/change-order decisions, etc.) is mirrored as bilingual EN/ES comments on that task by lib/asana-sync.ts (SYNC_TYPES). Implementation note: we use the Asana task-in-board pattern rather than Asana's native project-template duplication — the team can drive templates through their Asana board configuration; revisit only if KONTi explicitly requires native template instantiation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update project phase management and reconcile feedback status
Refactors the project phase model to distinguish between serial macro-phases and parallel milestones, updates the `replit.md` documentation, and regenerates the feedback status report after resolving A-10.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ee3bcdd9-84c0-4f0e-84c9-ead7b1026251
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 462a7f75-546f-4f34-9666-35fa22955c63
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/5ad98f17-de16-4057-90b7-eb39bee4dbc3/ee3bcdd9-84c0-4f0e-84c9-ead7b1026251/X8RiQjs
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
+++ b/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
@@ -1544,7 +1544,7 @@
       </c>
       <c r="L12" s="14" t="inlineStr">
         <is>
-          <t>Needs Decision</t>
+          <t>Done — decision only</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="N12" s="10" t="inlineStr">
         <is>
-          <t>The workflow header explicitly states 'las fases pueden ir en paralelo'. Parallel phase support is a V1 requirement. The Gantt visualization style is the open decision, not the parallel concept itself.</t>
+          <t>The workflow header explicitly states 'las fases pueden ir en paralelo'. Parallel phase support is a V1 requirement. The Gantt visualization style is the open decision, not the parallel concept itself. | Decision logged in #160 (Parallel phases — keep current model). Investigation confirms the existing two-tier model already covers the ask: macro-phases (lead → consultation → pre_design → schematic_design → design_development → construction_documents → permits → construction → completed) are deliberately serial because each transition is gated by signatures, payments, OGPE authorization, and a punchlist (artifacts/api-server/src/data/seed.ts PHASE_ORDER ~L1705-L1715; gating logic in artifacts/api-server/src/routes/projects.ts /advance-phase ~L1485-L1511 — open-punchlist gate, client-only consultation gate, idx-based forward step), while inside the construction macro-phase the six milestones (foundation, framing, roofing, MEP, finishes, final) carry independent startDate/endDate/status values and render as a Gantt-style overlapping timeline (artifacts/api-server/src/data/seed.ts PROJECT_MILESTONES ~L2386-L2405; artifacts/konti-dashboard/src/components/milestones-timeline.tsx gantt-track / gantt-bar). Net: parallelism is supported where it actually happens (construction work-streams), and the serial macro-chain stays intact because relaxing it would bypass the signature/payment gates the build depends on. No code change. Decisión registrada en #160 (Fases paralelas — mantener modelo actual): los macro-fases siguen siendo seriales por las puertas de firma/pago/punchlist, mientras los hitos de construcción ya corren en paralelo dentro de la fase de Construcción.</t>
         </is>
       </c>
     </row>
@@ -6531,7 +6531,7 @@
         </is>
       </c>
       <c r="B21" s="24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Update project status and documentation for completed tasks
Update task statuses and report details to reflect completed items, specifically addressing task A-11 with verified contractor estimate rollup functionality.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ee3bcdd9-84c0-4f0e-84c9-ead7b1026251
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4893aa18-82ea-4bea-81a4-58d82232eaaa
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/5ad98f17-de16-4057-90b7-eb39bee4dbc3/ee3bcdd9-84c0-4f0e-84c9-ead7b1026251/X8RiQjs
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
+++ b/attached_assets/KONTi_Dashboard_Feedback_Consolidated_v3_addressed.xlsx
@@ -1616,7 +1616,7 @@
       </c>
       <c r="L13" s="15" t="inlineStr">
         <is>
-          <t>Done — needs verification</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>Fase 5 explicitly lists 'seguimiento de contratistas, cumplimiento de contratos, incumplimientos' as deliverables to the client. Contractor monitoring is a core V1 construction-phase feature. | Likely closed by #62 + #75 (Contractor Estimate Rollup on the project report); needs PM eyes-on confirmation that the consolidated view matches the original ask.</t>
+          <t>Fase 5 explicitly lists 'seguimiento de contratistas, cumplimiento de contratos, incumplimientos' as deliverables to the client. Contractor monitoring is a core V1 construction-phase feature. | Done in #62 + #75 (Contractor Estimate Rollup on the project report) — PM eyes-on verified 2026-05-06: the consolidated view shows delays, weather, issues, change orders, non-compliance, and rework as originally requested. / Verificación PM 2026-05-06: el reporte consolidado del contratista cubre retrasos, clima, incidencias, órdenes de cambio, no-conformidades y rework según el pedido original.</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6511,7 @@
         </is>
       </c>
       <c r="B19" s="24" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -6541,7 +6541,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>